<commit_message>
add yanming into the group info
</commit_message>
<xml_diff>
--- a/STA380GroupForm.xlsx
+++ b/STA380GroupForm.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\STA380\STA380project\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{083E6859-A37D-4B1C-A7AC-C3882B2FD0C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="21960" windowHeight="12660"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="17253" windowHeight="10133" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,12 +28,15 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="51">
   <si>
     <t>If left blank, you will be assigned a number.</t>
   </si>
@@ -116,7 +125,7 @@
         <sz val="10"/>
         <color indexed="12"/>
         <rFont val="Arial"/>
-        <charset val="134"/>
+        <family val="2"/>
       </rPr>
       <t>https://github.com/CSJ111</t>
     </r>
@@ -140,7 +149,7 @@
         <sz val="10"/>
         <color indexed="12"/>
         <rFont val="Arial"/>
-        <charset val="134"/>
+        <family val="2"/>
       </rPr>
       <t>https://github.com/q1ngyao</t>
     </r>
@@ -179,7 +188,7 @@
         <sz val="10"/>
         <color indexed="12"/>
         <rFont val="Arial"/>
-        <charset val="134"/>
+        <family val="2"/>
       </rPr>
       <t>https://github.com/char1029</t>
     </r>
@@ -198,19 +207,24 @@
   </si>
   <si>
     <t>To report an inactive member, please refer to the "Reporting Inactive Members" section under the project description.</t>
+  </si>
+  <si>
+    <t>Yanming Zhao</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>zhaoy439</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://github.com/Yanming41</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="25">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -223,181 +237,49 @@
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="10"/>
       <color indexed="12"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Helvetica Neue"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Helvetica Neue"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Helvetica Neue"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Helvetica Neue"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Helvetica Neue"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Helvetica Neue"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -416,194 +298,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="19">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -725,253 +421,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1007,59 +464,15 @@
     <xf numFmtId="49" fontId="2" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="9" xfId="6" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+    <cellStyle name="超链接" xfId="1" builtinId="8"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
@@ -1132,6 +545,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1338,7 +754,7 @@
           <a:miter lim="800000"/>
         </a:ln>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1621,7 +1037,7 @@
           <a:miter lim="800000"/>
         </a:ln>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1897,7 +1313,7 @@
           <a:miter lim="400000"/>
         </a:ln>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -2170,25 +1586,26 @@
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultColWidth="12.5" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="12.46875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.5" style="1" customWidth="1"/>
+    <col min="1" max="1" width="31.46875" style="1" customWidth="1"/>
     <col min="2" max="2" width="76" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15.3482142857143" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.1696428571429" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.3482142857143" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="12.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.3515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.17578125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.46875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.3515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.46875" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="12.46875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:6">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1">
       <c r="A1" s="2"/>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -2198,7 +1615,7 @@
       <c r="E1" s="20"/>
       <c r="F1" s="14"/>
     </row>
-    <row r="2" customHeight="1" spans="1:6">
+    <row r="2" spans="1:6" ht="15.75" customHeight="1">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -2210,7 +1627,7 @@
       <c r="E2" s="14"/>
       <c r="F2" s="14"/>
     </row>
-    <row r="3" ht="13.65" customHeight="1" spans="1:6">
+    <row r="3" spans="1:6" ht="13.7" customHeight="1">
       <c r="A3" s="8"/>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -2218,7 +1635,7 @@
       <c r="E3" s="14"/>
       <c r="F3" s="14"/>
     </row>
-    <row r="4" customHeight="1" spans="1:6">
+    <row r="4" spans="1:6" ht="15.75" customHeight="1">
       <c r="A4" s="10"/>
       <c r="B4" s="11" t="s">
         <v>3</v>
@@ -2228,7 +1645,7 @@
       <c r="E4" s="20"/>
       <c r="F4" s="14"/>
     </row>
-    <row r="5" customHeight="1" spans="1:6">
+    <row r="5" spans="1:6" ht="15.75" customHeight="1">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -2240,7 +1657,7 @@
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
     </row>
-    <row r="6" customHeight="1" spans="1:6">
+    <row r="6" spans="1:6" ht="15.75" customHeight="1">
       <c r="A6" s="5" t="s">
         <v>6</v>
       </c>
@@ -2252,7 +1669,7 @@
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
     </row>
-    <row r="7" customHeight="1" spans="1:6">
+    <row r="7" spans="1:6" ht="15.75" customHeight="1">
       <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
@@ -2264,7 +1681,7 @@
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
     </row>
-    <row r="8" customHeight="1" spans="1:6">
+    <row r="8" spans="1:6" ht="15.75" customHeight="1">
       <c r="A8" s="16"/>
       <c r="B8" s="17"/>
       <c r="C8" s="14"/>
@@ -2272,7 +1689,7 @@
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
     </row>
-    <row r="9" customHeight="1" spans="1:6">
+    <row r="9" spans="1:6" ht="15.75" customHeight="1">
       <c r="A9" s="16"/>
       <c r="B9" s="18"/>
       <c r="C9" s="14"/>
@@ -2280,7 +1697,7 @@
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
     </row>
-    <row r="10" customHeight="1" spans="1:6">
+    <row r="10" spans="1:6" ht="15.75" customHeight="1">
       <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
@@ -2292,7 +1709,7 @@
       <c r="E10" s="14"/>
       <c r="F10" s="14"/>
     </row>
-    <row r="11" customHeight="1" spans="1:6">
+    <row r="11" spans="1:6" ht="15.75" customHeight="1">
       <c r="A11" s="5" t="s">
         <v>6</v>
       </c>
@@ -2304,7 +1721,7 @@
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
     </row>
-    <row r="12" customHeight="1" spans="1:6">
+    <row r="12" spans="1:6" ht="15.75" customHeight="1">
       <c r="A12" s="5" t="s">
         <v>8</v>
       </c>
@@ -2316,7 +1733,7 @@
       <c r="E12" s="14"/>
       <c r="F12" s="14"/>
     </row>
-    <row r="13" customHeight="1" spans="1:6">
+    <row r="13" spans="1:6" ht="15.75" customHeight="1">
       <c r="A13" s="16"/>
       <c r="B13" s="20"/>
       <c r="C13" s="14"/>
@@ -2324,7 +1741,7 @@
       <c r="E13" s="14"/>
       <c r="F13" s="14"/>
     </row>
-    <row r="14" customHeight="1" spans="1:6">
+    <row r="14" spans="1:6" ht="15.75" customHeight="1">
       <c r="A14" s="16"/>
       <c r="B14" s="20"/>
       <c r="C14" s="14"/>
@@ -2332,7 +1749,7 @@
       <c r="E14" s="14"/>
       <c r="F14" s="14"/>
     </row>
-    <row r="15" customHeight="1" spans="1:6">
+    <row r="15" spans="1:6" ht="15.75" customHeight="1">
       <c r="A15" s="5" t="s">
         <v>14</v>
       </c>
@@ -2344,7 +1761,7 @@
       <c r="E15" s="14"/>
       <c r="F15" s="14"/>
     </row>
-    <row r="16" customHeight="1" spans="1:6">
+    <row r="16" spans="1:6" ht="15.75" customHeight="1">
       <c r="A16" s="5" t="s">
         <v>6</v>
       </c>
@@ -2356,7 +1773,7 @@
       <c r="E16" s="14"/>
       <c r="F16" s="14"/>
     </row>
-    <row r="17" customHeight="1" spans="1:6">
+    <row r="17" spans="1:6" ht="15.75" customHeight="1">
       <c r="A17" s="5" t="s">
         <v>8</v>
       </c>
@@ -2368,7 +1785,7 @@
       <c r="E17" s="14"/>
       <c r="F17" s="14"/>
     </row>
-    <row r="18" customHeight="1" spans="1:6">
+    <row r="18" spans="1:6" ht="15.75" customHeight="1">
       <c r="A18" s="16"/>
       <c r="B18" s="20"/>
       <c r="C18" s="14"/>
@@ -2376,7 +1793,7 @@
       <c r="E18" s="14"/>
       <c r="F18" s="14"/>
     </row>
-    <row r="19" ht="13.65" customHeight="1" spans="1:6">
+    <row r="19" spans="1:6" ht="13.7" customHeight="1">
       <c r="A19" s="8"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
@@ -2384,7 +1801,7 @@
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" customHeight="1" spans="1:6">
+    <row r="20" spans="1:6" ht="15.75" customHeight="1">
       <c r="A20" s="10"/>
       <c r="B20" s="11" t="s">
         <v>18</v>
@@ -2402,7 +1819,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" customHeight="1" spans="1:6">
+    <row r="21" spans="1:6" ht="15.75" customHeight="1">
       <c r="A21" s="5" t="s">
         <v>23</v>
       </c>
@@ -2422,7 +1839,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="22" customHeight="1" spans="1:6">
+    <row r="22" spans="1:6" ht="15.75" customHeight="1">
       <c r="A22" s="5" t="s">
         <v>28</v>
       </c>
@@ -2442,7 +1859,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" customHeight="1" spans="1:6">
+    <row r="23" spans="1:6" ht="15.75" customHeight="1">
       <c r="A23" s="5" t="s">
         <v>33</v>
       </c>
@@ -2462,7 +1879,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" customHeight="1" spans="1:6">
+    <row r="24" spans="1:6" ht="15.75" customHeight="1">
       <c r="A24" s="5" t="s">
         <v>38</v>
       </c>
@@ -2482,17 +1899,27 @@
         <v>42</v>
       </c>
     </row>
-    <row r="25" customHeight="1" spans="1:6">
+    <row r="25" spans="1:6" ht="15.75" customHeight="1">
       <c r="A25" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B25" s="20"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-    </row>
-    <row r="26" ht="13.65" customHeight="1" spans="1:6">
+      <c r="B25" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="D25" s="14">
+        <v>1010452895</v>
+      </c>
+      <c r="E25" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="F25" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="13.7" customHeight="1">
       <c r="A26" s="7"/>
       <c r="B26" s="14"/>
       <c r="C26" s="14"/>
@@ -2500,7 +1927,7 @@
       <c r="E26" s="14"/>
       <c r="F26" s="14"/>
     </row>
-    <row r="27" customHeight="1" spans="1:6">
+    <row r="27" spans="1:6" ht="15.75" customHeight="1">
       <c r="A27" s="24" t="s">
         <v>44</v>
       </c>
@@ -2510,7 +1937,7 @@
       <c r="E27" s="14"/>
       <c r="F27" s="14"/>
     </row>
-    <row r="28" customHeight="1" spans="1:6">
+    <row r="28" spans="1:6" ht="15.75" customHeight="1">
       <c r="A28" s="24" t="s">
         <v>45</v>
       </c>
@@ -2520,7 +1947,7 @@
       <c r="E28" s="14"/>
       <c r="F28" s="14"/>
     </row>
-    <row r="29" customHeight="1" spans="1:6">
+    <row r="29" spans="1:6" ht="15.75" customHeight="1">
       <c r="A29" s="24" t="s">
         <v>46</v>
       </c>
@@ -2530,7 +1957,7 @@
       <c r="E29" s="14"/>
       <c r="F29" s="14"/>
     </row>
-    <row r="30" customHeight="1" spans="1:6">
+    <row r="30" spans="1:6" ht="15.75" customHeight="1">
       <c r="A30" s="24" t="s">
         <v>47</v>
       </c>
@@ -2541,14 +1968,15 @@
       <c r="F30" s="14"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="F21" r:id="rId1" display="https://github.com/CSJ111"/>
-    <hyperlink ref="F22" r:id="rId2" display="https://github.com/q1ngyao"/>
-    <hyperlink ref="F24" r:id="rId3" display="https://github.com/char1029"/>
-    <hyperlink ref="F23" r:id="rId4" display="https://github.com/DMZ66"/>
+    <hyperlink ref="F21" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F22" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F24" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F23" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait" useFirstPageNumber="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>